<commit_message>
Add Migration and Seeding
</commit_message>
<xml_diff>
--- a/public/templates/Form_IKU.xlsx
+++ b/public/templates/Form_IKU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghifa\Documents\admin-dashboard\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8860E05-072A-43A9-9C42-327B69074266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88BF72FB-A4D5-4722-955A-E51515612D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BFAE523-3C32-487F-867A-BFB50E6068E4}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>TARGET</t>
   </si>
@@ -73,13 +73,28 @@
   </si>
   <si>
     <t>PROGRAM KERJA</t>
+  </si>
+  <si>
+    <t>Mengetahui,</t>
+  </si>
+  <si>
+    <t>HC, FINANCE DIRECTORATE</t>
+  </si>
+  <si>
+    <t>Plt. Director</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Tempat, Tanggal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,7 +133,15 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
@@ -143,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -266,43 +289,6 @@
       </top>
       <bottom style="thin">
         <color theme="0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
       </bottom>
       <diagonal/>
     </border>
@@ -322,49 +308,69 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -372,24 +378,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -811,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5ED201A-4871-4AE9-AD96-2BD70DBEC7EB}">
-  <dimension ref="A3:M12"/>
+  <dimension ref="A3:M46"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
@@ -826,59 +814,58 @@
     <col min="10" max="10" width="11" style="1" customWidth="1"/>
     <col min="11" max="11" width="24" style="1" customWidth="1"/>
     <col min="12" max="12" width="17.5546875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="1"/>
+    <col min="13" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-    </row>
-    <row r="4" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-    </row>
-    <row r="5" spans="1:13" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-    </row>
-    <row r="6" spans="1:13" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+    </row>
+    <row r="4" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+    </row>
+    <row r="6" spans="1:12" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -891,100 +878,153 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-    </row>
-    <row r="8" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+    </row>
+    <row r="8" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="14"/>
+      <c r="E8" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="G8" s="27"/>
-      <c r="H8" s="22" t="s">
+      <c r="G8" s="18"/>
+      <c r="H8" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="I8" s="16" t="s">
+      <c r="I8" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="J8" s="17" t="s">
+      <c r="J8" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="K8" s="9" t="s">
+      <c r="K8" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="L8" s="12" t="s">
+      <c r="L8" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="M8" s="5"/>
-    </row>
-    <row r="9" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="5"/>
-    </row>
-    <row r="10" spans="1:13" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
+    </row>
+    <row r="9" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="24"/>
+    </row>
+    <row r="10" spans="1:12" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E10" s="21"/>
+      <c r="E10" s="27"/>
       <c r="F10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H10" s="22"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="7"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M12" s="6"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="19"/>
+    </row>
+    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B36" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="J36" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6"/>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B37" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B45" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="6"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="7"/>
+      <c r="M45" s="7"/>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="J46" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="K46" s="6"/>
+      <c r="L46" s="6"/>
+      <c r="M46" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="20">
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="L8:L10"/>
     <mergeCell ref="I8:I10"/>
     <mergeCell ref="J8:J10"/>
     <mergeCell ref="E8:E10"/>
     <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B3:J4"/>
+    <mergeCell ref="B5:J6"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="C8:D9"/>
     <mergeCell ref="F8:G9"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="B3:J4"/>
-    <mergeCell ref="B5:J6"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="J46:M46"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="J37:M37"/>
+    <mergeCell ref="J45:M45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>